<commit_message>
PMO: denser RACI column legend, full-width Ask form, B2C pack status.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/DigiThane_Kickoff_RACI_TMC.xlsx
+++ b/public/DigiThane_Kickoff_RACI_TMC.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="904" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="291">
   <si>
     <t>DigiThane 2.0</t>
   </si>
@@ -130,7 +130,7 @@
     <t>TMC</t>
   </si>
   <si>
-    <t>Thane Municipal Corporation — authority and data fiduciary</t>
+    <t>Thane Municipal Corporation</t>
   </si>
   <si>
     <t>RailTel</t>
@@ -148,37 +148,37 @@
     <t>PM</t>
   </si>
   <si>
-    <t>Project Manager — sole coordinator with TMC / RailTel / Smartrags</t>
+    <t>Project Manager</t>
   </si>
   <si>
     <t>Eng</t>
   </si>
   <si>
-    <t>Technical Lead — answers through the Project Manager</t>
+    <t>Technical Lead</t>
   </si>
   <si>
     <t>Dev</t>
   </si>
   <si>
-    <t>Development team — people named by job title on Delivery Roles</t>
+    <t>Development team</t>
   </si>
   <si>
     <t>Ops</t>
   </si>
   <si>
-    <t>DigiThane operations (merchant verification after go-live)</t>
+    <t>DigiThane operations (merchant verification)</t>
   </si>
   <si>
     <t>ERP</t>
   </si>
   <si>
-    <t>Municipal ERP vendors (Ascentech / ABM) — when APIs apply</t>
+    <t>Municipal ERP (Ascentech / ABM)</t>
   </si>
   <si>
     <t>PG</t>
   </si>
   <si>
-    <t>Common payment gateway vendor — when payments apply</t>
+    <t>Common payment gateway</t>
   </si>
   <si>
     <t>Notes</t>
@@ -193,7 +193,7 @@
     <t>Colours: Accountable = red, Responsible = green, Consulted = gold, Informed = blue, Not applicable = grey.</t>
   </si>
   <si>
-    <t>Delivery Roles lists job titles on this project. TMC, RailTel, and Smartrags write to the Project Manager only. Do not call engineers directly.</t>
+    <t>Delivery Roles lists job titles on this project.</t>
   </si>
   <si>
     <t>Where municipal or payment-gateway documents are still awaited, those vendors stay Consulted until the documents arrive.</t>
@@ -283,19 +283,7 @@
     <t>Common payment gateway (G-06)</t>
   </si>
   <si>
-    <t>Merchant onboarding (G-10)</t>
-  </si>
-  <si>
-    <t>Merchant app (G-13)</t>
-  </si>
-  <si>
-    <t>Citizen marketplace bridge (G-12)</t>
-  </si>
-  <si>
-    <t>Advertisement packages (G-34)</t>
-  </si>
-  <si>
-    <t>Offers and coupons (G-11)</t>
+    <t>B2C pack — merchants, marketplace, ads, offers, classifieds, events, jobs, halls, premium, parking, property, tourism, clinics, daily deals (G-10, G-11, G-12, G-13, G-34, G-35, G-37, G-38, G-40, G-41, G-42, G-44, G-45, G-46, G-47)</t>
   </si>
   <si>
     <t>Forums (G-14)</t>
@@ -307,36 +295,6 @@
     <t>City alerts (G-09)</t>
   </si>
   <si>
-    <t>Classifieds (G-35)</t>
-  </si>
-  <si>
-    <t>Events / tickets (G-37)</t>
-  </si>
-  <si>
-    <t>Jobs (G-38)</t>
-  </si>
-  <si>
-    <t>Hall / ground booking (G-40)</t>
-  </si>
-  <si>
-    <t>Premium / ad-free (G-41)</t>
-  </si>
-  <si>
-    <t>Parking (G-42)</t>
-  </si>
-  <si>
-    <t>Property listings (G-44)</t>
-  </si>
-  <si>
-    <t>Tourism (G-45)</t>
-  </si>
-  <si>
-    <t>Clinic appointments (G-46)</t>
-  </si>
-  <si>
-    <t>Daily deals (G-47)</t>
-  </si>
-  <si>
     <t>Maps (G-17 / G-29)</t>
   </si>
   <si>
@@ -424,6 +382,18 @@
     <t>Security Engineer</t>
   </si>
   <si>
+    <t>UI</t>
+  </si>
+  <si>
+    <t>UI prototyping (Figma Make) — citizen and merchant screens</t>
+  </si>
+  <si>
+    <t>UI Designer</t>
+  </si>
+  <si>
+    <t>19 Aug 2026</t>
+  </si>
+  <si>
     <t>T+4</t>
   </si>
   <si>
@@ -523,61 +493,22 @@
     <t>G-06</t>
   </si>
   <si>
-    <t>Common payment gateway</t>
-  </si>
-  <si>
     <t>Integration Engineer, Backend Engineer</t>
   </si>
   <si>
     <t>When payment documents arrive</t>
   </si>
   <si>
-    <t>G-10</t>
-  </si>
-  <si>
-    <t>Merchant onboarding</t>
-  </si>
-  <si>
-    <t>G-13</t>
-  </si>
-  <si>
-    <t>Merchant app</t>
-  </si>
-  <si>
-    <t>Mobile Engineer, Backend Engineer</t>
-  </si>
-  <si>
-    <t>G-12</t>
-  </si>
-  <si>
-    <t>Citizen marketplace</t>
-  </si>
-  <si>
-    <t>Product Manager, Web Engineer, Mobile Engineer</t>
-  </si>
-  <si>
-    <t>G-34</t>
-  </si>
-  <si>
-    <t>Advertisement packages</t>
-  </si>
-  <si>
-    <t>Product Manager, Backend Engineer</t>
-  </si>
-  <si>
-    <t>After marketplace</t>
-  </si>
-  <si>
-    <t>G-11</t>
-  </si>
-  <si>
-    <t>Offers and coupons</t>
-  </si>
-  <si>
-    <t>Backend Engineer, Mobile Engineer</t>
-  </si>
-  <si>
-    <t>With merchant app</t>
+    <t>B2C</t>
+  </si>
+  <si>
+    <t>B2C pack — G-10 merchants, G-13 merchant app, G-12 marketplace, G-34 ads, G-11 offers, G-35 classifieds, G-37 events, G-38 jobs, G-40 halls, G-41 premium, G-42 parking, G-44 property, G-45 tourism, G-46 clinics, G-47 deals</t>
+  </si>
+  <si>
+    <t>Product Manager, Backend Engineer, Web Engineer, Mobile Engineer, Ops</t>
+  </si>
+  <si>
+    <t>UAT window</t>
   </si>
   <si>
     <t>G-14</t>
@@ -586,9 +517,6 @@
     <t>Forums</t>
   </si>
   <si>
-    <t>UAT window</t>
-  </si>
-  <si>
     <t>G-15</t>
   </si>
   <si>
@@ -604,66 +532,6 @@
     <t>City alerts</t>
   </si>
   <si>
-    <t>G-35</t>
-  </si>
-  <si>
-    <t>Classifieds</t>
-  </si>
-  <si>
-    <t>G-37</t>
-  </si>
-  <si>
-    <t>Events and tickets</t>
-  </si>
-  <si>
-    <t>G-38</t>
-  </si>
-  <si>
-    <t>Jobs</t>
-  </si>
-  <si>
-    <t>G-40</t>
-  </si>
-  <si>
-    <t>Hall and ground booking</t>
-  </si>
-  <si>
-    <t>G-41</t>
-  </si>
-  <si>
-    <t>Premium (advertisement-free commercial)</t>
-  </si>
-  <si>
-    <t>G-42</t>
-  </si>
-  <si>
-    <t>Parking</t>
-  </si>
-  <si>
-    <t>G-44</t>
-  </si>
-  <si>
-    <t>Property listings</t>
-  </si>
-  <si>
-    <t>G-45</t>
-  </si>
-  <si>
-    <t>Tourism</t>
-  </si>
-  <si>
-    <t>G-46</t>
-  </si>
-  <si>
-    <t>Clinic appointments</t>
-  </si>
-  <si>
-    <t>G-47</t>
-  </si>
-  <si>
-    <t>Daily deals</t>
-  </si>
-  <si>
     <t>G-17</t>
   </si>
   <si>
@@ -817,19 +685,13 @@
     <t>Mandate</t>
   </si>
   <si>
-    <t>Sets build order, accepts each module, raises blockers to the Project Manager</t>
-  </si>
-  <si>
-    <t>Project Manager</t>
-  </si>
-  <si>
-    <t>Single point of contact for TMC, RailTel, and Smartrags</t>
-  </si>
-  <si>
-    <t>Technical Lead</t>
-  </si>
-  <si>
-    <t>Day-to-day technical decisions and answers to written questions</t>
+    <t>Sets build order and accepts each module</t>
+  </si>
+  <si>
+    <t>Delivery plan, gates, and written questions</t>
+  </si>
+  <si>
+    <t>Day-to-day technical decisions</t>
   </si>
   <si>
     <t>Business Analyst</t>
@@ -916,10 +778,7 @@
     <t>Handover notes, design document support, operating notes</t>
   </si>
   <si>
-    <t>UI Designer</t>
-  </si>
-  <si>
-    <t>Screens in Marathi and English</t>
+    <t>Screen prototypes (Figma Make) and production UI in Marathi and English</t>
   </si>
   <si>
     <t>Communication SLA</t>
@@ -931,10 +790,10 @@
     <t>Commitment</t>
   </si>
   <si>
-    <t>Client contact path</t>
-  </si>
-  <si>
-    <t>Please write to the Project Manager only. The Technical Lead answers through the Project Manager. Team members are not available for direct calls or meetings.</t>
+    <t>PMO questions</t>
+  </si>
+  <si>
+    <t>Ask the Development Cell on the published board. Recorded in Netlify Forms.</t>
   </si>
   <si>
     <t>Acknowledge a question</t>
@@ -952,7 +811,7 @@
     <t>How the PMO board is updated</t>
   </si>
   <si>
-    <t>How this board is updated: at the end of each working day (IST) the Development Cell refreshes status, copies it into the public PMO site, and pushes git. Netlify rebuilds this page. The Excel file has no live status.</t>
+    <t>Updated: Everyday EOD (IST) Status Is Refreshed By Development Cell</t>
   </si>
   <si>
     <t>Board refresh target</t>
@@ -991,7 +850,16 @@
     <t>T+8 Proof of concept</t>
   </si>
   <si>
-    <t>Login, home, master control centre</t>
+    <t>Login, home, master control centre. Screen prototypes already done (Figma Make).</t>
+  </si>
+  <si>
+    <t>B2C pack</t>
+  </si>
+  <si>
+    <t>After MCC → UAT</t>
+  </si>
+  <si>
+    <t>One stream: merchants, marketplace, ads, offers, classifieds, events, jobs, halls, premium, parking, property, tourism, clinics, deals.</t>
   </si>
   <si>
     <t>UAT 1</t>
@@ -1909,7 +1777,7 @@
     <tabColor rgb="FFC1121F"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J57"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="48" customWidth="1"/>
@@ -2566,8 +2434,8 @@
       <c r="A24" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B24" s="20" t="s">
-        <v>29</v>
+      <c r="B24" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="C24" s="19" t="s">
         <v>26</v>
@@ -2590,16 +2458,16 @@
       <c r="I24" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="J24" s="20" t="s">
-        <v>29</v>
+      <c r="J24" s="18" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="B25" s="20" t="s">
-        <v>29</v>
+      <c r="B25" s="19" t="s">
+        <v>26</v>
       </c>
       <c r="C25" s="19" t="s">
         <v>26</v>
@@ -2616,22 +2484,22 @@
       <c r="G25" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="H25" s="17" t="s">
-        <v>20</v>
+      <c r="H25" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="I25" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="J25" s="18" t="s">
-        <v>23</v>
+      <c r="J25" s="20" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="B26" s="19" t="s">
-        <v>26</v>
+      <c r="B26" s="16" t="s">
+        <v>17</v>
       </c>
       <c r="C26" s="19" t="s">
         <v>26</v>
@@ -2642,28 +2510,28 @@
       <c r="E26" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F26" s="16" t="s">
-        <v>17</v>
+      <c r="F26" s="17" t="s">
+        <v>20</v>
       </c>
       <c r="G26" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="H26" s="18" t="s">
-        <v>23</v>
+      <c r="H26" s="20" t="s">
+        <v>29</v>
       </c>
       <c r="I26" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="J26" s="18" t="s">
-        <v>23</v>
+      <c r="J26" s="20" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="B27" s="18" t="s">
-        <v>23</v>
+      <c r="B27" s="16" t="s">
+        <v>17</v>
       </c>
       <c r="C27" s="19" t="s">
         <v>26</v>
@@ -2674,14 +2542,14 @@
       <c r="E27" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F27" s="16" t="s">
-        <v>17</v>
+      <c r="F27" s="17" t="s">
+        <v>20</v>
       </c>
       <c r="G27" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="H27" s="18" t="s">
-        <v>23</v>
+      <c r="H27" s="20" t="s">
+        <v>29</v>
       </c>
       <c r="I27" s="20" t="s">
         <v>29</v>
@@ -2694,8 +2562,8 @@
       <c r="A28" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B28" s="20" t="s">
-        <v>29</v>
+      <c r="B28" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="C28" s="19" t="s">
         <v>26</v>
@@ -2712,14 +2580,14 @@
       <c r="G28" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="H28" s="18" t="s">
-        <v>23</v>
+      <c r="H28" s="20" t="s">
+        <v>29</v>
       </c>
       <c r="I28" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="J28" s="18" t="s">
-        <v>23</v>
+      <c r="J28" s="20" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
@@ -2744,8 +2612,8 @@
       <c r="G29" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="H29" s="18" t="s">
-        <v>23</v>
+      <c r="H29" s="20" t="s">
+        <v>29</v>
       </c>
       <c r="I29" s="20" t="s">
         <v>29</v>
@@ -2758,26 +2626,26 @@
       <c r="A30" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="B30" s="16" t="s">
+      <c r="B30" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C30" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D30" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="E30" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F30" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C30" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D30" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E30" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F30" s="17" t="s">
-        <v>20</v>
-      </c>
       <c r="G30" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="H30" s="20" t="s">
-        <v>29</v>
+      <c r="H30" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="I30" s="20" t="s">
         <v>29</v>
@@ -2790,26 +2658,26 @@
       <c r="A31" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="B31" s="16" t="s">
+      <c r="B31" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C31" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="E31" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F31" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C31" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D31" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E31" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F31" s="17" t="s">
-        <v>20</v>
-      </c>
       <c r="G31" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="H31" s="20" t="s">
-        <v>29</v>
+      <c r="H31" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="I31" s="20" t="s">
         <v>29</v>
@@ -2818,65 +2686,47 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="23" t="s">
+    <row r="32" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="22" t="s">
         <v>95</v>
       </c>
-      <c r="B32" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="C32" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D32" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E32" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F32" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="G32" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="H32" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="I32" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="J32" s="20" t="s">
-        <v>29</v>
-      </c>
+      <c r="B32" s="22"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="I32" s="22"/>
+      <c r="J32" s="22"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="B33" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="C33" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D33" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E33" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F33" s="16" t="s">
+      <c r="B33" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="G33" s="17" t="s">
-        <v>20</v>
+      <c r="C33" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D33" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="E33" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F33" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="G33" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="H33" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="I33" s="20" t="s">
-        <v>29</v>
+      <c r="I33" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="J33" s="18" t="s">
         <v>23</v>
@@ -2886,61 +2736,61 @@
       <c r="A34" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="B34" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="C34" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D34" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E34" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F34" s="16" t="s">
+      <c r="B34" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="G34" s="17" t="s">
-        <v>20</v>
+      <c r="C34" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D34" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="E34" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F34" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="G34" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="H34" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="I34" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="J34" s="20" t="s">
-        <v>29</v>
+      <c r="I34" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="J34" s="18" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="B35" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C35" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D35" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E35" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F35" s="16" t="s">
+      <c r="B35" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="G35" s="17" t="s">
-        <v>20</v>
+      <c r="C35" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D35" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="E35" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F35" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="G35" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="H35" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="I35" s="20" t="s">
-        <v>29</v>
+      <c r="I35" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="J35" s="18" t="s">
         <v>23</v>
@@ -2950,21 +2800,21 @@
       <c r="A36" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="B36" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="C36" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D36" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E36" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F36" s="16" t="s">
+      <c r="B36" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C36" s="16" t="s">
         <v>17</v>
       </c>
+      <c r="D36" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="E36" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F36" s="18" t="s">
+        <v>23</v>
+      </c>
       <c r="G36" s="17" t="s">
         <v>20</v>
       </c>
@@ -2974,8 +2824,8 @@
       <c r="I36" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="J36" s="18" t="s">
-        <v>23</v>
+      <c r="J36" s="20" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
@@ -2985,18 +2835,18 @@
       <c r="B37" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="C37" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D37" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E37" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F37" s="16" t="s">
+      <c r="C37" s="16" t="s">
         <v>17</v>
       </c>
+      <c r="D37" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="E37" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F37" s="18" t="s">
+        <v>23</v>
+      </c>
       <c r="G37" s="17" t="s">
         <v>20</v>
       </c>
@@ -3006,22 +2856,22 @@
       <c r="I37" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="J37" s="18" t="s">
-        <v>23</v>
+      <c r="J37" s="20" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="B38" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="C38" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D38" s="20" t="s">
-        <v>29</v>
+      <c r="B38" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C38" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D38" s="19" t="s">
+        <v>26</v>
       </c>
       <c r="E38" s="18" t="s">
         <v>23</v>
@@ -3032,69 +2882,69 @@
       <c r="G38" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="H38" s="18" t="s">
-        <v>23</v>
+      <c r="H38" s="20" t="s">
+        <v>29</v>
       </c>
       <c r="I38" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="J38" s="18" t="s">
-        <v>23</v>
+      <c r="J38" s="20" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="B39" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C39" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D39" s="20" t="s">
-        <v>29</v>
+      <c r="B39" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D39" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="E39" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F39" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="G39" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="H39" s="18" t="s">
-        <v>23</v>
+      <c r="F39" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="G39" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="H39" s="20" t="s">
+        <v>29</v>
       </c>
       <c r="I39" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="J39" s="18" t="s">
-        <v>23</v>
+      <c r="J39" s="20" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="B40" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="C40" s="19" t="s">
-        <v>26</v>
+      <c r="B40" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C40" s="18" t="s">
+        <v>23</v>
       </c>
       <c r="D40" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="E40" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F40" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="G40" s="17" t="s">
-        <v>20</v>
+      <c r="E40" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F40" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="G40" s="19" t="s">
+        <v>26</v>
       </c>
       <c r="H40" s="18" t="s">
         <v>23</v>
@@ -3102,8 +2952,8 @@
       <c r="I40" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="J40" s="18" t="s">
-        <v>23</v>
+      <c r="J40" s="20" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
@@ -3128,37 +2978,37 @@
       <c r="G41" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="H41" s="18" t="s">
-        <v>23</v>
+      <c r="H41" s="20" t="s">
+        <v>29</v>
       </c>
       <c r="I41" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="J41" s="18" t="s">
-        <v>23</v>
+      <c r="J41" s="20" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="B42" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C42" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D42" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E42" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F42" s="16" t="s">
+      <c r="B42" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="G42" s="17" t="s">
-        <v>20</v>
+      <c r="C42" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D42" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="E42" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F42" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="G42" s="19" t="s">
+        <v>26</v>
       </c>
       <c r="H42" s="20" t="s">
         <v>29</v>
@@ -3174,461 +3024,31 @@
       <c r="A43" s="23" t="s">
         <v>106</v>
       </c>
-      <c r="B43" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="C43" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D43" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E43" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F43" s="16" t="s">
+      <c r="B43" s="16" t="s">
         <v>17</v>
       </c>
+      <c r="C43" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D43" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="E43" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F43" s="17" t="s">
+        <v>20</v>
+      </c>
       <c r="G43" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="H43" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="I43" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="J43" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A44" s="23" t="s">
-        <v>107</v>
-      </c>
-      <c r="B44" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C44" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D44" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E44" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F44" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="G44" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="H44" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="I44" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="J44" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A45" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="B45" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C45" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D45" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E45" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F45" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="G45" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="H45" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="I45" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="J45" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="46" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A46" s="22" t="s">
-        <v>109</v>
-      </c>
-      <c r="B46" s="22"/>
-      <c r="C46" s="22"/>
-      <c r="D46" s="22"/>
-      <c r="E46" s="22"/>
-      <c r="F46" s="22"/>
-      <c r="G46" s="22"/>
-      <c r="H46" s="22"/>
-      <c r="I46" s="22"/>
-      <c r="J46" s="22"/>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A47" s="23" t="s">
-        <v>110</v>
-      </c>
-      <c r="B47" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C47" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="D47" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="E47" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="F47" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="G47" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H47" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="I47" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="J47" s="18" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A48" s="23" t="s">
-        <v>111</v>
-      </c>
-      <c r="B48" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C48" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="D48" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="E48" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="F48" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="G48" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H48" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="I48" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="J48" s="18" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A49" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="B49" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C49" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="D49" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="E49" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="F49" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="G49" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H49" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="I49" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="J49" s="18" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A50" s="23" t="s">
-        <v>113</v>
-      </c>
-      <c r="B50" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C50" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="D50" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="E50" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="F50" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="G50" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="H50" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="I50" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="J50" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A51" s="23" t="s">
-        <v>114</v>
-      </c>
-      <c r="B51" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C51" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="D51" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="E51" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="F51" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="G51" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="H51" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="I51" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="J51" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A52" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="B52" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="C52" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="D52" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="E52" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F52" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="G52" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="H52" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="I52" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="J52" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A53" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="B53" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="C53" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="D53" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="E53" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F53" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="G53" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="H53" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="I53" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="J53" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A54" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="B54" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="C54" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="D54" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E54" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="F54" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="G54" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="H54" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="I54" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="J54" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A55" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="B55" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="C55" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D55" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E55" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="F55" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="G55" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="H55" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="I55" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="J55" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A56" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="B56" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C56" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="D56" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="E56" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="F56" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="G56" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="H56" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="I56" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="J56" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A57" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="B57" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C57" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="D57" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="E57" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="F57" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="G57" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="H57" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="I57" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="J57" s="19" t="s">
+      <c r="H43" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="I43" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="J43" s="19" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3639,7 +3059,7 @@
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A6:J6"/>
     <mergeCell ref="A20:J20"/>
-    <mergeCell ref="A46:J46"/>
+    <mergeCell ref="A32:J32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
@@ -3651,7 +3071,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -3663,7 +3083,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -3679,271 +3099,271 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>123</v>
+        <v>109</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="23" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="C5" s="23" t="s">
         <v>75</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="23" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>137</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="23" t="s">
+        <v>113</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="E7" s="23" t="s">
         <v>127</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>138</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>139</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="23" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="23" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="23" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="23" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="23" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>152</v>
+        <v>80</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>153</v>
+        <v>140</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="23" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>156</v>
+        <v>143</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>157</v>
+        <v>138</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="23" t="s">
-        <v>158</v>
+        <v>113</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="23" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="23" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>166</v>
+        <v>153</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>167</v>
+        <v>154</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>168</v>
+        <v>116</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="B17" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="C17" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>157</v>
+      </c>
+      <c r="E17" s="23" t="s">
         <v>158</v>
-      </c>
-      <c r="B17" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="C17" s="23" t="s">
-        <v>171</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>156</v>
-      </c>
-      <c r="E17" s="23" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="23" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>173</v>
+        <v>160</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>174</v>
+        <v>161</v>
       </c>
       <c r="E18" s="23" t="s">
         <v>162</v>
@@ -3951,16 +3371,16 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="23" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>177</v>
+        <v>151</v>
       </c>
       <c r="E19" s="23" t="s">
         <v>162</v>
@@ -3968,512 +3388,291 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="23" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>178</v>
+        <v>165</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>179</v>
+        <v>166</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>180</v>
+        <v>167</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>181</v>
+        <v>162</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="23" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>182</v>
+        <v>168</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>183</v>
+        <v>169</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>184</v>
+        <v>129</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>185</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="23" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>186</v>
+        <v>170</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>187</v>
+        <v>171</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>188</v>
+        <v>162</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="23" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>188</v>
+        <v>162</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="23" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>193</v>
+        <v>177</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>139</v>
+        <v>178</v>
       </c>
       <c r="E24" s="23" t="s">
-        <v>188</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="23" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>177</v>
+        <v>151</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>188</v>
+        <v>162</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="23" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>197</v>
+        <v>182</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>188</v>
+        <v>162</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="23" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>188</v>
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="23" t="s">
-        <v>158</v>
+        <v>186</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>200</v>
+        <v>187</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>201</v>
+        <v>188</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>161</v>
+        <v>189</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="23" t="s">
-        <v>158</v>
+        <v>186</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="C29" s="23" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>139</v>
+        <v>189</v>
       </c>
       <c r="E29" s="23" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="23" t="s">
-        <v>158</v>
+        <v>186</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>161</v>
+        <v>189</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="23" t="s">
-        <v>158</v>
+        <v>186</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="C31" s="23" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>177</v>
+        <v>199</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="23" t="s">
-        <v>158</v>
+        <v>186</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>177</v>
+        <v>199</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="23" t="s">
-        <v>158</v>
+        <v>186</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="C33" s="23" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>161</v>
+        <v>205</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>188</v>
+        <v>206</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
-        <v>158</v>
+        <v>186</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="D34" s="23" t="s">
-        <v>177</v>
+        <v>209</v>
       </c>
       <c r="E34" s="23" t="s">
-        <v>188</v>
+        <v>210</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="23" t="s">
-        <v>158</v>
+        <v>186</v>
       </c>
       <c r="B35" s="23" t="s">
+        <v>211</v>
+      </c>
+      <c r="C35" s="23" t="s">
+        <v>212</v>
+      </c>
+      <c r="D35" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="E35" s="23" t="s">
         <v>214</v>
-      </c>
-      <c r="C35" s="23" t="s">
-        <v>215</v>
-      </c>
-      <c r="D35" s="23" t="s">
-        <v>216</v>
-      </c>
-      <c r="E35" s="23" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="23" t="s">
-        <v>158</v>
+        <v>186</v>
       </c>
       <c r="B36" s="23" t="s">
+        <v>215</v>
+      </c>
+      <c r="C36" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="D36" s="23" t="s">
+        <v>216</v>
+      </c>
+      <c r="E36" s="23" t="s">
         <v>217</v>
-      </c>
-      <c r="C36" s="23" t="s">
-        <v>218</v>
-      </c>
-      <c r="D36" s="23" t="s">
-        <v>219</v>
-      </c>
-      <c r="E36" s="23" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="23" t="s">
-        <v>158</v>
-      </c>
-      <c r="B37" s="23" t="s">
-        <v>220</v>
-      </c>
-      <c r="C37" s="23" t="s">
-        <v>221</v>
-      </c>
-      <c r="D37" s="23" t="s">
-        <v>222</v>
-      </c>
-      <c r="E37" s="23" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="23" t="s">
-        <v>158</v>
-      </c>
-      <c r="B38" s="23" t="s">
-        <v>223</v>
-      </c>
-      <c r="C38" s="23" t="s">
-        <v>224</v>
-      </c>
-      <c r="D38" s="23" t="s">
-        <v>161</v>
-      </c>
-      <c r="E38" s="23" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="23" t="s">
-        <v>158</v>
-      </c>
-      <c r="B39" s="23" t="s">
-        <v>225</v>
-      </c>
-      <c r="C39" s="23" t="s">
-        <v>226</v>
-      </c>
-      <c r="D39" s="23" t="s">
-        <v>156</v>
-      </c>
-      <c r="E39" s="23" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="23" t="s">
-        <v>158</v>
-      </c>
-      <c r="B40" s="23" t="s">
-        <v>227</v>
-      </c>
-      <c r="C40" s="23" t="s">
-        <v>228</v>
-      </c>
-      <c r="D40" s="23" t="s">
-        <v>229</v>
-      </c>
-      <c r="E40" s="23" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="23" t="s">
-        <v>230</v>
-      </c>
-      <c r="B41" s="23" t="s">
-        <v>231</v>
-      </c>
-      <c r="C41" s="23" t="s">
-        <v>232</v>
-      </c>
-      <c r="D41" s="23" t="s">
-        <v>233</v>
-      </c>
-      <c r="E41" s="23" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="23" t="s">
-        <v>230</v>
-      </c>
-      <c r="B42" s="23" t="s">
-        <v>235</v>
-      </c>
-      <c r="C42" s="23" t="s">
-        <v>236</v>
-      </c>
-      <c r="D42" s="23" t="s">
-        <v>233</v>
-      </c>
-      <c r="E42" s="23" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="23" t="s">
-        <v>230</v>
-      </c>
-      <c r="B43" s="23" t="s">
-        <v>238</v>
-      </c>
-      <c r="C43" s="23" t="s">
-        <v>239</v>
-      </c>
-      <c r="D43" s="23" t="s">
-        <v>233</v>
-      </c>
-      <c r="E43" s="23" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="23" t="s">
-        <v>230</v>
-      </c>
-      <c r="B44" s="23" t="s">
-        <v>241</v>
-      </c>
-      <c r="C44" s="23" t="s">
-        <v>242</v>
-      </c>
-      <c r="D44" s="23" t="s">
-        <v>243</v>
-      </c>
-      <c r="E44" s="23" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="23" t="s">
-        <v>230</v>
-      </c>
-      <c r="B45" s="23" t="s">
-        <v>245</v>
-      </c>
-      <c r="C45" s="23" t="s">
-        <v>246</v>
-      </c>
-      <c r="D45" s="23" t="s">
-        <v>243</v>
-      </c>
-      <c r="E45" s="23" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="23" t="s">
-        <v>230</v>
-      </c>
-      <c r="B46" s="23" t="s">
-        <v>247</v>
-      </c>
-      <c r="C46" s="23" t="s">
-        <v>248</v>
-      </c>
-      <c r="D46" s="23" t="s">
-        <v>249</v>
-      </c>
-      <c r="E46" s="23" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="23" t="s">
-        <v>230</v>
-      </c>
-      <c r="B47" s="23" t="s">
-        <v>251</v>
-      </c>
-      <c r="C47" s="23" t="s">
-        <v>252</v>
-      </c>
-      <c r="D47" s="23" t="s">
-        <v>253</v>
-      </c>
-      <c r="E47" s="23" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="23" t="s">
-        <v>230</v>
-      </c>
-      <c r="B48" s="23" t="s">
-        <v>255</v>
-      </c>
-      <c r="C48" s="23" t="s">
-        <v>256</v>
-      </c>
-      <c r="D48" s="23" t="s">
-        <v>257</v>
-      </c>
-      <c r="E48" s="23" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="23" t="s">
-        <v>230</v>
-      </c>
-      <c r="B49" s="23" t="s">
-        <v>259</v>
-      </c>
-      <c r="C49" s="23" t="s">
-        <v>2</v>
-      </c>
-      <c r="D49" s="23" t="s">
-        <v>260</v>
-      </c>
-      <c r="E49" s="23" t="s">
-        <v>261</v>
       </c>
     </row>
   </sheetData>
@@ -4495,7 +3694,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>262</v>
+        <v>218</v>
       </c>
       <c r="B1" s="15"/>
     </row>
@@ -4505,170 +3704,170 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
-        <v>263</v>
+        <v>219</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>264</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="23" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>265</v>
+        <v>221</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
-        <v>266</v>
+        <v>42</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>267</v>
+        <v>222</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="23" t="s">
-        <v>268</v>
+        <v>44</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>269</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="23" t="s">
-        <v>270</v>
+        <v>224</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>271</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="23" t="s">
-        <v>272</v>
+        <v>226</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>273</v>
+        <v>227</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="23" t="s">
-        <v>274</v>
+        <v>228</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>275</v>
+        <v>229</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="23" t="s">
-        <v>276</v>
+        <v>230</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>277</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="23" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>278</v>
+        <v>232</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="23" t="s">
-        <v>279</v>
+        <v>233</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>280</v>
+        <v>234</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="23" t="s">
-        <v>281</v>
+        <v>235</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>282</v>
+        <v>236</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="23" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>283</v>
+        <v>237</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="23" t="s">
-        <v>284</v>
+        <v>238</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>285</v>
+        <v>239</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="23" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>286</v>
+        <v>240</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="23" t="s">
-        <v>287</v>
+        <v>241</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>288</v>
+        <v>242</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="23" t="s">
-        <v>289</v>
+        <v>243</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>290</v>
+        <v>244</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="23" t="s">
-        <v>291</v>
+        <v>245</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>292</v>
+        <v>246</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="23" t="s">
-        <v>293</v>
+        <v>247</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>294</v>
+        <v>248</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="23" t="s">
-        <v>222</v>
+        <v>178</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>295</v>
+        <v>249</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="23" t="s">
-        <v>296</v>
+        <v>250</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>297</v>
+        <v>251</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="23" t="s">
-        <v>298</v>
+        <v>122</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>299</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -4690,7 +3889,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>300</v>
+        <v>253</v>
       </c>
       <c r="B1" s="15"/>
     </row>
@@ -4700,50 +3899,50 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
-        <v>301</v>
+        <v>254</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>302</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="23" t="s">
-        <v>303</v>
+        <v>256</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>304</v>
+        <v>257</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
-        <v>305</v>
+        <v>258</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>306</v>
+        <v>259</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="23" t="s">
-        <v>307</v>
+        <v>260</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>308</v>
+        <v>261</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="23" t="s">
-        <v>309</v>
+        <v>262</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>310</v>
+        <v>263</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="23" t="s">
-        <v>311</v>
+        <v>264</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>312</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -4756,7 +3955,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -4766,7 +3965,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>313</v>
+        <v>266</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -4778,112 +3977,123 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
-        <v>314</v>
+        <v>267</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>315</v>
+        <v>268</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>316</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="23" t="s">
-        <v>317</v>
+        <v>270</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>318</v>
+        <v>271</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>319</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
-        <v>320</v>
+        <v>273</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>321</v>
+        <v>274</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="23" t="s">
-        <v>322</v>
+        <v>275</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>323</v>
+        <v>276</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="23" t="s">
-        <v>324</v>
+        <v>277</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>234</v>
+        <v>278</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>325</v>
+        <v>279</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="23" t="s">
-        <v>326</v>
+        <v>280</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>237</v>
+        <v>190</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>327</v>
+        <v>281</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="23" t="s">
-        <v>328</v>
+        <v>282</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>240</v>
+        <v>193</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>329</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="23" t="s">
-        <v>330</v>
+        <v>284</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>244</v>
+        <v>196</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>331</v>
+        <v>285</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="23" t="s">
-        <v>332</v>
+        <v>286</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>258</v>
+        <v>200</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>333</v>
+        <v>287</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="23" t="s">
+        <v>288</v>
+      </c>
+      <c r="B12" s="23" t="s">
+        <v>214</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="23" t="s">
-        <v>261</v>
-      </c>
-      <c r="C12" s="23" t="s">
-        <v>334</v>
+      <c r="B13" s="23" t="s">
+        <v>217</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>290</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PMO: trim column legend, drop Figma Make wording, chat-style threads.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/DigiThane_Kickoff_RACI_TMC.xlsx
+++ b/public/DigiThane_Kickoff_RACI_TMC.xlsx
@@ -385,7 +385,7 @@
     <t>UI</t>
   </si>
   <si>
-    <t>UI prototyping (Figma Make) — citizen and merchant screens</t>
+    <t>UI prototyping — citizen and merchant screens</t>
   </si>
   <si>
     <t>UI Designer</t>
@@ -778,7 +778,7 @@
     <t>Handover notes, design document support, operating notes</t>
   </si>
   <si>
-    <t>Screen prototypes (Figma Make) and production UI in Marathi and English</t>
+    <t>Screen prototypes and production UI in Marathi and English</t>
   </si>
   <si>
     <t>Communication SLA</t>
@@ -850,7 +850,7 @@
     <t>T+8 Proof of concept</t>
   </si>
   <si>
-    <t>Login, home, master control centre. Screen prototypes already done (Figma Make).</t>
+    <t>Login, home, master control centre. Screen prototypes already done.</t>
   </si>
   <si>
     <t>B2C pack</t>

</xml_diff>